<commit_message>
Apply red-team fixes across the package
Fix unverified surgery-site and clinic claims, competitor overstatement,
add cost per contact, state an exclusivity position, align the rubric,
bidding ladder, gates, and CPC ranges across files, set document
metadata, and tighten the note to Kristina. Adds the QA report.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GD6g2VXLwfea8fyRm3LH8N
</commit_message>
<xml_diff>
--- a/hartigan-ppc/04_budget_model.xlsx
+++ b/hartigan-ppc/04_budget_model.xlsx
@@ -1327,7 +1327,7 @@
     <t xml:space="preserve">Pre-launch</t>
   </si>
   <si>
-    <t xml:space="preserve">Days -14 to 0</t>
+    <t xml:space="preserve">Days -28 to 0</t>
   </si>
   <si>
     <t xml:space="preserve">Practice confirms intake phone hours (placeholder Monday to Friday, 8 am to 5 pm Central), the navigation and robotic systems and facilities (O12), and whether TCO marketing must approve. Vendor BAAs signed (call tracking, forms); DNI number and form event built; landing pages live; negative list loaded; campaigns built but paused.</t>
@@ -1450,7 +1450,7 @@
     <t xml:space="preserve">Search impression share, lost to budget, and lost to rank read from Google Ads for each campaign.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lost to rank above lost to budget means the demand cap is real: hold the cap. Lost to budget above 20% means demand exceeds the model: raise the cap in $500 steps at day 60.</t>
+    <t xml:space="preserve">Lost to rank above lost to budget means the demand cap is real: hold the cap. Lost to budget above 10% means demand exceeds the model: raise the cap in $500 steps between day 60 and day 90.</t>
   </si>
   <si>
     <t xml:space="preserve">modeled achievable impression share</t>
@@ -1770,151 +1770,151 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2180,22 +2180,22 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -2229,7 +2229,7 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>11</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
         <v>15</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>16</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>18</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>19</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>20</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
         <v>21</v>
       </c>
@@ -2378,7 +2378,7 @@
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>22</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
         <v>25</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>26</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>27</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>28</v>
       </c>
@@ -2493,7 +2493,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>29</v>
       </c>
@@ -2516,7 +2516,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
         <v>30</v>
       </c>
@@ -2527,7 +2527,7 @@
       <c r="F20" s="6"/>
       <c r="G20" s="6"/>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>35</v>
       </c>
@@ -2573,7 +2573,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
         <v>39</v>
       </c>
@@ -2584,7 +2584,7 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
         <v>40</v>
       </c>
@@ -2607,7 +2607,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
         <v>44</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
         <v>45</v>
       </c>
@@ -2653,7 +2653,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
         <v>46</v>
       </c>
@@ -2664,7 +2664,7 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
         <v>47</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>51</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
         <v>52</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
         <v>53</v>
       </c>
@@ -2744,7 +2744,7 @@
       <c r="F31" s="6"/>
       <c r="G31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
         <v>54</v>
       </c>
@@ -2767,7 +2767,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
         <v>58</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
         <v>59</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
         <v>60</v>
       </c>
@@ -2836,7 +2836,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>61</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>62</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>63</v>
       </c>
@@ -2905,7 +2905,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>65</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>66</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
         <v>67</v>
       </c>
@@ -2974,7 +2974,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
         <v>68</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
         <v>69</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>70</v>
       </c>
@@ -3043,7 +3043,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
         <v>72</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
         <v>73</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>74</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>75</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>76</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>77</v>
       </c>
@@ -3169,7 +3169,7 @@
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
     </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>78</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>82</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>85</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
         <v>88</v>
       </c>
@@ -3261,7 +3261,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
         <v>91</v>
       </c>
@@ -3272,7 +3272,7 @@
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
     </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>92</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>96</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
         <v>97</v>
       </c>
@@ -3341,7 +3341,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
         <v>98</v>
       </c>
@@ -3352,7 +3352,7 @@
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
     </row>
-    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>99</v>
       </c>
@@ -3375,7 +3375,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
         <v>103</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
         <v>104</v>
       </c>
@@ -3421,7 +3421,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
         <v>105</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
         <v>106</v>
       </c>
@@ -3467,7 +3467,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
         <v>107</v>
       </c>
@@ -3490,7 +3490,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
         <v>108</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
         <v>109</v>
       </c>
@@ -3536,7 +3536,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
         <v>110</v>
       </c>
@@ -3559,7 +3559,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
         <v>111</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
         <v>112</v>
       </c>
@@ -3605,7 +3605,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
         <v>113</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
         <v>114</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
         <v>115</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
         <v>116</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
         <v>117</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
         <v>118</v>
       </c>
@@ -3743,7 +3743,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
         <v>119</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
         <v>120</v>
       </c>
@@ -3777,7 +3777,7 @@
       <c r="F78" s="6"/>
       <c r="G78" s="6"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
         <v>121</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
         <v>125</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
         <v>128</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
         <v>132</v>
       </c>
@@ -3902,7 +3902,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
         <v>135</v>
       </c>
@@ -3946,7 +3946,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
         <v>149</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
         <v>149</v>
       </c>
@@ -4034,7 +4034,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
         <v>149</v>
       </c>
@@ -4078,7 +4078,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>149</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>149</v>
       </c>
@@ -4166,7 +4166,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
         <v>149</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
         <v>149</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
         <v>149</v>
       </c>
@@ -4298,7 +4298,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
         <v>149</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
         <v>149</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
         <v>149</v>
       </c>
@@ -4430,7 +4430,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
         <v>149</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>149</v>
       </c>
@@ -4518,7 +4518,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
         <v>149</v>
       </c>
@@ -4562,7 +4562,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
         <v>149</v>
       </c>
@@ -4606,7 +4606,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>149</v>
       </c>
@@ -4650,7 +4650,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>149</v>
       </c>
@@ -4694,7 +4694,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>149</v>
       </c>
@@ -4738,7 +4738,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>149</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>149</v>
       </c>
@@ -4826,7 +4826,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>149</v>
       </c>
@@ -4870,7 +4870,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>149</v>
       </c>
@@ -4914,7 +4914,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
         <v>149</v>
       </c>
@@ -4958,7 +4958,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
         <v>149</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
         <v>149</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
         <v>212</v>
       </c>
@@ -5090,7 +5090,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
         <v>212</v>
       </c>
@@ -5134,7 +5134,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>212</v>
       </c>
@@ -5178,7 +5178,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
         <v>212</v>
       </c>
@@ -5222,7 +5222,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>212</v>
       </c>
@@ -5266,7 +5266,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
         <v>212</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
         <v>212</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
         <v>212</v>
       </c>
@@ -5398,7 +5398,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
         <v>212</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
         <v>212</v>
       </c>
@@ -5486,7 +5486,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>212</v>
       </c>
@@ -5530,7 +5530,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>212</v>
       </c>
@@ -5574,7 +5574,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>212</v>
       </c>
@@ -5618,7 +5618,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>212</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
         <v>212</v>
       </c>
@@ -5706,7 +5706,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
         <v>212</v>
       </c>
@@ -5750,7 +5750,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
         <v>212</v>
       </c>
@@ -5794,7 +5794,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
         <v>212</v>
       </c>
@@ -5838,7 +5838,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
         <v>212</v>
       </c>
@@ -5882,7 +5882,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
         <v>212</v>
       </c>
@@ -5926,7 +5926,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>212</v>
       </c>
@@ -5970,7 +5970,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>212</v>
       </c>
@@ -6014,7 +6014,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>212</v>
       </c>
@@ -6058,7 +6058,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>212</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>212</v>
       </c>
@@ -6146,7 +6146,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>212</v>
       </c>
@@ -6190,7 +6190,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
         <v>212</v>
       </c>
@@ -6234,7 +6234,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
         <v>266</v>
       </c>
@@ -6278,7 +6278,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>266</v>
       </c>
@@ -6322,7 +6322,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>266</v>
       </c>
@@ -6366,7 +6366,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>266</v>
       </c>
@@ -6410,7 +6410,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
         <v>266</v>
       </c>
@@ -6454,7 +6454,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
         <v>266</v>
       </c>
@@ -6498,7 +6498,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>266</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
         <v>266</v>
       </c>
@@ -6586,7 +6586,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
         <v>266</v>
       </c>
@@ -6630,7 +6630,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
         <v>266</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
         <v>266</v>
       </c>
@@ -6718,7 +6718,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
         <v>266</v>
       </c>
@@ -6762,7 +6762,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
         <v>266</v>
       </c>
@@ -6806,7 +6806,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
         <v>266</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
         <v>266</v>
       </c>
@@ -6894,7 +6894,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
         <v>266</v>
       </c>
@@ -6938,7 +6938,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
         <v>266</v>
       </c>
@@ -6982,7 +6982,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
         <v>266</v>
       </c>
@@ -7026,7 +7026,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
         <v>266</v>
       </c>
@@ -7070,7 +7070,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
         <v>266</v>
       </c>
@@ -7114,7 +7114,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
         <v>266</v>
       </c>
@@ -7158,7 +7158,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
         <v>311</v>
       </c>
@@ -7202,7 +7202,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
         <v>311</v>
       </c>
@@ -7246,7 +7246,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
         <v>311</v>
       </c>
@@ -7290,7 +7290,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
         <v>311</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
         <v>311</v>
       </c>
@@ -7378,7 +7378,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
         <v>311</v>
       </c>
@@ -7422,7 +7422,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
         <v>311</v>
       </c>
@@ -7466,7 +7466,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
         <v>311</v>
       </c>
@@ -7510,7 +7510,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
         <v>311</v>
       </c>
@@ -7554,7 +7554,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
         <v>311</v>
       </c>
@@ -7598,7 +7598,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
         <v>311</v>
       </c>
@@ -7642,7 +7642,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
         <v>311</v>
       </c>
@@ -7686,7 +7686,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
         <v>335</v>
       </c>
@@ -7730,7 +7730,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
         <v>335</v>
       </c>
@@ -7774,7 +7774,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
         <v>335</v>
       </c>
@@ -7818,7 +7818,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
         <v>335</v>
       </c>
@@ -7862,7 +7862,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
         <v>335</v>
       </c>
@@ -7906,7 +7906,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
         <v>335</v>
       </c>
@@ -7950,7 +7950,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
         <v>335</v>
       </c>
@@ -7994,7 +7994,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
         <v>335</v>
       </c>
@@ -8038,7 +8038,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
         <v>335</v>
       </c>
@@ -8082,7 +8082,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
         <v>335</v>
       </c>
@@ -8126,7 +8126,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
         <v>335</v>
       </c>
@@ -8170,7 +8170,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
         <v>358</v>
       </c>
@@ -8214,7 +8214,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
         <v>358</v>
       </c>
@@ -8258,7 +8258,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
         <v>358</v>
       </c>
@@ -8302,7 +8302,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
         <v>358</v>
       </c>
@@ -8346,7 +8346,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
         <v>358</v>
       </c>
@@ -8390,7 +8390,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
         <v>358</v>
       </c>
@@ -8434,7 +8434,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
         <v>358</v>
       </c>
@@ -8478,7 +8478,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
         <v>358</v>
       </c>
@@ -8522,7 +8522,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
         <v>358</v>
       </c>
@@ -8566,7 +8566,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
         <v>358</v>
       </c>
@@ -8610,7 +8610,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
         <v>358</v>
       </c>
@@ -8654,7 +8654,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
         <v>358</v>
       </c>
@@ -8698,7 +8698,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
         <v>358</v>
       </c>
@@ -8773,12 +8773,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="16" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>382</v>
       </c>
@@ -8827,7 +8827,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
         <v>397</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>1018.51851851852</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
         <v>397</v>
       </c>
@@ -8939,7 +8939,7 @@
         <v>395.952957404051</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
         <v>397</v>
       </c>
@@ -8995,7 +8995,7 @@
         <v>250.140463491037</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
         <v>398</v>
       </c>
@@ -9051,7 +9051,7 @@
         <v>973.172711350336</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
         <v>398</v>
       </c>
@@ -9107,7 +9107,7 @@
         <v>396.446954083462</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
         <v>398</v>
       </c>
@@ -9163,7 +9163,7 @@
         <v>260.255144680021</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
         <v>399</v>
       </c>
@@ -9219,7 +9219,7 @@
         <v>1040.22241781578</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
         <v>399</v>
       </c>
@@ -9275,7 +9275,7 @@
         <v>426.830058859263</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
         <v>399</v>
       </c>
@@ -9331,12 +9331,12 @@
         <v>282.458051358116</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
         <v>401</v>
       </c>
@@ -9414,7 +9414,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
         <v>410</v>
       </c>
@@ -9487,7 +9487,7 @@
         <v>1037.03703703704</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>411</v>
       </c>
@@ -9560,7 +9560,7 @@
         <v>1037.03703703704</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
         <v>412</v>
       </c>
@@ -9633,7 +9633,7 @@
         <v>740.740740740741</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
         <v>312</v>
       </c>
@@ -9706,7 +9706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
         <v>413</v>
       </c>
@@ -9779,7 +9779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
         <v>414</v>
       </c>
@@ -9852,7 +9852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
         <v>415</v>
       </c>
@@ -9925,7 +9925,7 @@
         <v>1018.51851851852</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
         <v>416</v>
       </c>
@@ -10003,7 +10003,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
         <v>410</v>
       </c>
@@ -10076,7 +10076,7 @@
         <v>402.212166918049</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
         <v>411</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>402.212166918049</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
         <v>412</v>
       </c>
@@ -10222,7 +10222,7 @@
         <v>321.769733534439</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
         <v>312</v>
       </c>
@@ -10295,7 +10295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
         <v>413</v>
       </c>
@@ -10368,7 +10368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
         <v>414</v>
       </c>
@@ -10441,7 +10441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="25" t="s">
         <v>415</v>
       </c>
@@ -10514,7 +10514,7 @@
         <v>395.952957404051</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
         <v>417</v>
       </c>
@@ -10592,7 +10592,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
         <v>410</v>
       </c>
@@ -10665,7 +10665,7 @@
         <v>258.79917184265</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
         <v>411</v>
       </c>
@@ -10738,7 +10738,7 @@
         <v>258.79917184265</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
         <v>412</v>
       </c>
@@ -10811,7 +10811,7 @@
         <v>210.274327122153</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
         <v>312</v>
       </c>
@@ -10884,7 +10884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
         <v>413</v>
       </c>
@@ -10957,7 +10957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
         <v>414</v>
       </c>
@@ -11030,7 +11030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="25" t="s">
         <v>415</v>
       </c>
@@ -11103,7 +11103,7 @@
         <v>250.140463491037</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>418</v>
       </c>
@@ -11181,7 +11181,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
         <v>410</v>
       </c>
@@ -11254,7 +11254,7 @@
         <v>1140.74074074074</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
         <v>411</v>
       </c>
@@ -11327,7 +11327,7 @@
         <v>1140.74074074074</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
         <v>412</v>
       </c>
@@ -11400,7 +11400,7 @@
         <v>814.814814814815</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
         <v>312</v>
       </c>
@@ -11473,7 +11473,7 @@
         <v>814.814814814815</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>413</v>
       </c>
@@ -11546,7 +11546,7 @@
         <v>651.851851851852</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
         <v>414</v>
       </c>
@@ -11619,7 +11619,7 @@
         <v>814.814814814815</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="25" t="s">
         <v>415</v>
       </c>
@@ -11692,7 +11692,7 @@
         <v>973.172711350336</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
         <v>419</v>
       </c>
@@ -11770,7 +11770,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>410</v>
       </c>
@@ -11843,7 +11843,7 @@
         <v>442.433383609854</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
         <v>411</v>
       </c>
@@ -11916,7 +11916,7 @@
         <v>442.433383609854</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
         <v>412</v>
       </c>
@@ -11989,7 +11989,7 @@
         <v>353.946706887883</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
         <v>312</v>
       </c>
@@ -12062,7 +12062,7 @@
         <v>353.946706887883</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
         <v>413</v>
       </c>
@@ -12135,7 +12135,7 @@
         <v>309.703368526898</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
         <v>414</v>
       </c>
@@ -12208,7 +12208,7 @@
         <v>353.946706887883</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="25" t="s">
         <v>415</v>
       </c>
@@ -12281,7 +12281,7 @@
         <v>396.446954083462</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
         <v>420</v>
       </c>
@@ -12359,7 +12359,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
         <v>410</v>
       </c>
@@ -12432,7 +12432,7 @@
         <v>284.679089026915</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
         <v>411</v>
       </c>
@@ -12505,7 +12505,7 @@
         <v>284.679089026915</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
         <v>412</v>
       </c>
@@ -12578,7 +12578,7 @@
         <v>231.301759834369</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
         <v>312</v>
       </c>
@@ -12651,7 +12651,7 @@
         <v>231.301759834368</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
         <v>413</v>
       </c>
@@ -12724,7 +12724,7 @@
         <v>213.509316770186</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
         <v>414</v>
       </c>
@@ -12797,7 +12797,7 @@
         <v>231.301759834369</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="25" t="s">
         <v>415</v>
       </c>
@@ -12870,7 +12870,7 @@
         <v>260.255144680021</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
         <v>421</v>
       </c>
@@ -12948,7 +12948,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
         <v>410</v>
       </c>
@@ -13021,7 +13021,7 @@
         <v>1244.44444444444</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
         <v>411</v>
       </c>
@@ -13094,7 +13094,7 @@
         <v>1244.44444444444</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
         <v>412</v>
       </c>
@@ -13167,7 +13167,7 @@
         <v>888.888888888889</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
         <v>312</v>
       </c>
@@ -13240,7 +13240,7 @@
         <v>888.888888888889</v>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
         <v>413</v>
       </c>
@@ -13313,7 +13313,7 @@
         <v>711.111111111111</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
         <v>414</v>
       </c>
@@ -13386,7 +13386,7 @@
         <v>888.888888888889</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="25" t="s">
         <v>415</v>
       </c>
@@ -13459,7 +13459,7 @@
         <v>1040.22241781578</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="5" t="s">
         <v>422</v>
       </c>
@@ -13537,7 +13537,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
         <v>410</v>
       </c>
@@ -13610,7 +13610,7 @@
         <v>482.654600301659</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
         <v>411</v>
       </c>
@@ -13683,7 +13683,7 @@
         <v>482.654600301659</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
         <v>412</v>
       </c>
@@ -13756,7 +13756,7 @@
         <v>386.123680241327</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
         <v>312</v>
       </c>
@@ -13829,7 +13829,7 @@
         <v>386.123680241327</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
         <v>413</v>
       </c>
@@ -13902,7 +13902,7 @@
         <v>337.858220211161</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
         <v>414</v>
       </c>
@@ -13975,7 +13975,7 @@
         <v>386.123680241327</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="25" t="s">
         <v>415</v>
       </c>
@@ -14048,7 +14048,7 @@
         <v>426.830058859263</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="5" t="s">
         <v>423</v>
       </c>
@@ -14126,7 +14126,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
         <v>410</v>
       </c>
@@ -14199,7 +14199,7 @@
         <v>310.55900621118</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
         <v>411</v>
       </c>
@@ -14272,7 +14272,7 @@
         <v>310.55900621118</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
         <v>412</v>
       </c>
@@ -14345,7 +14345,7 @@
         <v>252.329192546584</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
         <v>312</v>
       </c>
@@ -14418,7 +14418,7 @@
         <v>252.329192546584</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
         <v>413</v>
       </c>
@@ -14491,7 +14491,7 @@
         <v>232.919254658385</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
         <v>414</v>
       </c>
@@ -14564,7 +14564,7 @@
         <v>252.329192546584</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="25" t="s">
         <v>415</v>
       </c>
@@ -14666,17 +14666,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>426</v>
       </c>
@@ -14702,7 +14702,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
         <v>433</v>
       </c>
@@ -14724,7 +14724,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="33" t="s">
         <v>439</v>
       </c>
@@ -14751,7 +14751,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
         <v>439</v>
       </c>
@@ -14778,7 +14778,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
         <v>439</v>
       </c>
@@ -14805,7 +14805,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
         <v>452</v>
       </c>
@@ -14827,7 +14827,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
         <v>458</v>
       </c>
@@ -14854,7 +14854,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
         <v>458</v>
       </c>
@@ -14881,7 +14881,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
         <v>458</v>
       </c>
@@ -14908,7 +14908,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
         <v>458</v>
       </c>
@@ -14935,7 +14935,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
         <v>473</v>
       </c>
@@ -14962,7 +14962,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="33" t="s">
         <v>477</v>
       </c>
@@ -14989,7 +14989,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="33" t="s">
         <v>481</v>
       </c>
@@ -15016,7 +15016,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
         <v>481</v>
       </c>
@@ -15043,7 +15043,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="33" t="s">
         <v>486</v>
       </c>
@@ -15070,7 +15070,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="33" t="s">
         <v>486</v>
       </c>
@@ -15097,7 +15097,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="s">
         <v>486</v>
       </c>
@@ -15124,7 +15124,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="s">
         <v>486</v>
       </c>
@@ -15151,7 +15151,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="33" t="s">
         <v>486</v>
       </c>
@@ -15178,7 +15178,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="33" t="s">
         <v>486</v>
       </c>
@@ -15205,7 +15205,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="33" t="s">
         <v>486</v>
       </c>
@@ -15232,7 +15232,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="33" t="s">
         <v>505</v>
       </c>
@@ -15259,7 +15259,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="33" t="s">
         <v>505</v>
       </c>
@@ -15286,7 +15286,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="33" t="s">
         <v>505</v>
       </c>
@@ -15313,7 +15313,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="33" t="s">
         <v>505</v>
       </c>
@@ -15340,7 +15340,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="33" t="s">
         <v>505</v>
       </c>
@@ -15367,7 +15367,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="33" t="s">
         <v>505</v>
       </c>
@@ -15394,7 +15394,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="33" t="s">
         <v>505</v>
       </c>
@@ -15421,7 +15421,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="33" t="s">
         <v>505</v>
       </c>
@@ -15448,7 +15448,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
         <v>505</v>
       </c>
@@ -15475,7 +15475,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
         <v>505</v>
       </c>

</xml_diff>

<commit_message>
Add the ppc-research-proposal skill
Reusable multi-agent workflow for Google Ads research-to-proposal runs:
SKILL.md orchestration, agent brief templates, standards, compliance
modules by vertical, proposal structure, lessons from the Hartigan run,
and scripts for the docx and md builder, package quality gate, sources
merge, and environment check.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GD6g2VXLwfea8fyRm3LH8N
</commit_message>
<xml_diff>
--- a/hartigan-ppc/04_budget_model.xlsx
+++ b/hartigan-ppc/04_budget_model.xlsx
@@ -1770,151 +1770,151 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>